<commit_message>
Atualiza catalogo para Dia das Maes 2026 e publica nova colecao
</commit_message>
<xml_diff>
--- a/data/produtos.xlsx
+++ b/data/produtos.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Velas\02_Site\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CBD588C-7AAD-4C8A-B2CB-17105D6460D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BA4C07B-04D3-481B-BA83-4B53F906555D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Produtos" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="123">
   <si>
     <t>ativo</t>
   </si>
@@ -118,156 +131,21 @@
     <t>nao</t>
   </si>
   <si>
-    <t>vela-aromatica-ambar-belluno-essenza</t>
-  </si>
-  <si>
-    <t>Vela Aromática Âmbar Belluno Essenza</t>
-  </si>
-  <si>
-    <t>Elegância sensorial em vidro âmbar</t>
-  </si>
-  <si>
     <t>Velas aromáticas</t>
   </si>
   <si>
-    <t>Amadeirada oriental</t>
-  </si>
-  <si>
-    <t>200 g</t>
-  </si>
-  <si>
     <t>40 horas</t>
   </si>
   <si>
-    <t>Vela aromática sofisticada em vidro âmbar que perfuma o ambiente com elegância.</t>
-  </si>
-  <si>
-    <t>A vela aromática Belluno Essenza em copo de vidro âmbar combina design sofisticado com uma fragrância envolvente e acolhedora. Sua composição cria uma atmosfera elegante e relaxante, ideal para momentos de descanso ou para valorizar ambientes refinados. O vidro âmbar e a tampa dourada conferem um toque contemporâneo e luxuoso à decoração.</t>
-  </si>
-  <si>
-    <t>Bergamota, laranja doce</t>
-  </si>
-  <si>
-    <t>Âmbar, jasmim, cedro</t>
-  </si>
-  <si>
-    <t>Baunilha, sândalo, musk</t>
-  </si>
-  <si>
-    <t>Acenda sobre superfície resistente ao calor e deixe queimar até formar uma piscina uniforme de cera.</t>
-  </si>
-  <si>
-    <t>Cera vegetal premium, fragrância fina, pavio de algodão, copo de vidro âmbar, tampa metálica dourada</t>
-  </si>
-  <si>
-    <t>vela-aromatica-ambar-belluno-essenza.png</t>
-  </si>
-  <si>
-    <t>BE-VA-AMB-200</t>
-  </si>
-  <si>
-    <t>Vela Aromática Âmbar Belluno Essenza | Vela Premium em Vidro Âmbar</t>
-  </si>
-  <si>
-    <t>Vela aromática premium Belluno Essenza em vidro âmbar com fragrância sofisticada e design elegante para perfumar e decorar ambientes com estilo.</t>
-  </si>
-  <si>
-    <t>vela-aromatica-vidro-transparente-madeira-belluno</t>
-  </si>
-  <si>
-    <t>Velas Belluno Essenza Lumière</t>
-  </si>
-  <si>
-    <t>Vidro transparente com tampa de madeira natural</t>
-  </si>
-  <si>
     <t>Floral amadeirada</t>
   </si>
   <si>
-    <t>220 g</t>
-  </si>
-  <si>
     <t>45 horas</t>
   </si>
   <si>
-    <t>Vela aromática premium em vidro transparente espesso com acabamento elegante e fragrância envolvente.</t>
-  </si>
-  <si>
-    <t>A vela Belluno Essenza Lumière combina design minimalista com uma fragrância sofisticada que transforma o ambiente em um espaço acolhedor e elegante. Produzida com cera cremosa de alta qualidade e pavio central para queima uniforme, ela é apresentada em um copo de vidro transparente espesso com tampa de madeira clara natural. Sua fragrância delicada cria uma atmosfera relaxante e refinada para momentos especiais. Ideal para compor ambientes sofisticados e rituais de bem-estar.</t>
-  </si>
-  <si>
-    <t>Bergamota, pêra, mandarina</t>
-  </si>
-  <si>
-    <t>Jasmim, flor de laranjeira, lírio branco</t>
-  </si>
-  <si>
-    <t>Sândalo, baunilha, musk branco</t>
-  </si>
-  <si>
-    <t>Acenda sobre superfície resistente ao calor e mantenha a vela acesa sob supervisão.</t>
-  </si>
-  <si>
-    <t>Cera vegetal premium, fragrância fina, pavio de algodão, recipiente de vidro espesso, tampa de madeira natural</t>
-  </si>
-  <si>
-    <t>vela-aromatica-vidro-transparente-madeira-belluno.png</t>
-  </si>
-  <si>
-    <t>BEL-VE-002</t>
-  </si>
-  <si>
-    <t>Vela Aromática Premium Belluno Essenza Lumière em Vidro Transparente</t>
-  </si>
-  <si>
-    <t>Vela aromática premium Belluno Essenza em vidro transparente com tampa de madeira natural e fragrância sofisticada para ambientes elegantes.</t>
-  </si>
-  <si>
-    <t>vela-ceramica-off-white-belluno-essenza</t>
-  </si>
-  <si>
-    <t>Vela Aromática Belluno Essenza Cerâmica Off-White</t>
-  </si>
-  <si>
-    <t>Elegância minimalista em cerâmica artesanal</t>
-  </si>
-  <si>
     <t>Floral amadeirada suave</t>
   </si>
   <si>
-    <t>Uma vela sofisticada em cerâmica fosca que perfuma o ambiente com elegância e suavidade.</t>
-  </si>
-  <si>
-    <t>Produzida artesanalmente, esta vela Belluno Essenza apresenta recipiente de cerâmica fosca off-white com design minimalista e refinado, ideal para ambientes elegantes e acolhedores. Sua fragrância floral amadeirada cria uma atmosfera sofisticada e relaxante. A peça também funciona como elemento decorativo atemporal, elevando a estética do espaço.</t>
-  </si>
-  <si>
-    <t>Bergamota, limão siciliano</t>
-  </si>
-  <si>
-    <t>Jasmim, flor de algodão</t>
-  </si>
-  <si>
-    <t>Sândalo, musk branco, âmbar</t>
-  </si>
-  <si>
-    <t>Acenda sobre superfície resistente ao calor e deixe a cera derreter até as bordas na primeira queima para melhor desempenho.</t>
-  </si>
-  <si>
-    <t>Cera vegetal premium, fragrância fina, pavio de algodão, recipiente de cerâmica fosca</t>
-  </si>
-  <si>
-    <t>vela-ceramica-off-white-belluno-essenza.png</t>
-  </si>
-  <si>
-    <t>BE-CER-220OW</t>
-  </si>
-  <si>
-    <t>Vela Aromática Belluno Essenza em Cerâmica Off-White Premium</t>
-  </si>
-  <si>
-    <t>Vela aromática premium em recipiente de cerâmica fosca off-white com fragrância floral amadeirada elegante, ideal para criar ambientes sofisticados e acolhedores.</t>
-  </si>
-  <si>
     <t>vela-aromatica-lata-nude-belluno</t>
   </si>
   <si>
@@ -461,13 +339,76 @@
   </si>
   <si>
     <t>Vela aromática premium Belluno Essenza em elegante recipiente de vidro canelado com fragrância floral sofisticada e design decorativo refinado.</t>
+  </si>
+  <si>
+    <t>vela-aromatica-belluno-essenza-dia-das-maes</t>
+  </si>
+  <si>
+    <t>Vela Aromática Coleção Dia Das Mães 2026</t>
+  </si>
+  <si>
+    <t>Presentei a pessoa que você mais ama</t>
+  </si>
+  <si>
+    <t>Coleção dia das Mães 2026</t>
+  </si>
+  <si>
+    <t>60g</t>
+  </si>
+  <si>
+    <t>12 horas</t>
+  </si>
+  <si>
+    <t>Vela aromática artesanal da Coleção Dia das Mães, criada para presentear com delicadeza, perfume suave e acabamento elegante.</t>
+  </si>
+  <si>
+    <t>A Vela Aromática Belluno Essenza Coleção Dia das Mães 2026 foi desenvolvida para transformar o ato de presentear em uma lembrança delicada e sofisticada. Produzida artesanalmente, combina cera vegetal premium, pavio de algodão e fragrância floral suave com fundo levemente amadeirado, criando uma atmosfera acolhedora sem excesso. Seu acabamento clean valoriza a decoração e torna a peça ideal para kits presenteáveis, mesas de apoio, lavabos, quartos e pequenos ambientes. Uma escolha elegante para demonstrar carinho com perfume, luz e presença.</t>
+  </si>
+  <si>
+    <t>Bergamota, limão siciliano, chá branco</t>
+  </si>
+  <si>
+    <t>Jasmim, flor de algodão, peônia delicada</t>
+  </si>
+  <si>
+    <t>Sândalo, musk branco, âmbar suave</t>
+  </si>
+  <si>
+    <t>Cera vegetal premium, essência aromática fina, pavio de algodão e recipiente decorativo.</t>
+  </si>
+  <si>
+    <t>vela-dia-das-maes-belluno-essenza.png</t>
+  </si>
+  <si>
+    <t>vela-dia-das-maes-belluno-essenza-01.png</t>
+  </si>
+  <si>
+    <t>vela-dia-das-maes-belluno-essenza-02.png</t>
+  </si>
+  <si>
+    <t>vela-dia-das-maes-belluno-essenza-03.png</t>
+  </si>
+  <si>
+    <t>BE-DMAES-60G-2026</t>
+  </si>
+  <si>
+    <t>Edição especial Dia das Mães</t>
+  </si>
+  <si>
+    <t>Vela Aromática Dia das Mães Belluno Essenza | Presente Artesanal</t>
+  </si>
+  <si>
+    <t>Vela aromática artesanal Belluno Essenza da Coleção Dia das Mães, com fragrância floral suave, acabamento elegante e proposta delicada para presentear.</t>
+  </si>
+  <si>
+    <t>Use sobre superfície plana e resistente ao calor. Na primeira queima, deixe a cera derreter até próximo das bordas para evitar túnel. Nunca use sem supervisão.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -480,6 +421,12 @@
       <sz val="11"/>
       <color rgb="FFF7F2EA"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -519,10 +466,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -533,9 +481,13 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{018ABC54-90D8-4F39-A81B-E354B1AF4273}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -835,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB8"/>
+  <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -949,325 +901,329 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" ht="116" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C2" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>32</v>
+        <v>102</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>33</v>
+        <v>103</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>34</v>
+        <v>104</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I2" s="3">
-        <v>29.9</v>
-      </c>
-      <c r="J2" s="3">
-        <v>22.9</v>
-      </c>
+        <v>32.9</v>
+      </c>
+      <c r="J2" s="3"/>
       <c r="K2" s="2" t="s">
-        <v>37</v>
+        <v>106</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="U2" s="2"/>
-      <c r="V2" s="2"/>
-      <c r="W2" s="2"/>
-      <c r="X2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y2" s="2">
-        <v>42</v>
-      </c>
-      <c r="Z2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="W2" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="X2" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y2" s="4">
         <v>30</v>
       </c>
-      <c r="AA2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>49</v>
+      <c r="Z2" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="AA2" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="AB2" s="4" t="s">
+        <v>121</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C3" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="I3" s="3">
-        <v>21.9</v>
+        <v>42.9</v>
       </c>
       <c r="J3" s="3"/>
       <c r="K3" s="2" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
       <c r="W3" s="2"/>
       <c r="X3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y3" s="2">
         <v>64</v>
-      </c>
-      <c r="Y3" s="2">
-        <v>32</v>
       </c>
       <c r="Z3" s="2" t="s">
         <v>30</v>
       </c>
       <c r="AA3" s="2" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="AB3" s="2" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" ht="87" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C4" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="I4" s="3">
-        <v>37.9</v>
+        <v>29.9</v>
       </c>
       <c r="J4" s="3">
-        <v>31.9</v>
+        <v>19.899999999999999</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
       <c r="X4" s="2" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="Y4" s="2">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="Z4" s="2" t="s">
         <v>29</v>
       </c>
       <c r="AA4" s="2" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="AB4" s="2" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C5" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="I5" s="3">
-        <v>42.9</v>
+        <v>34.99</v>
       </c>
       <c r="J5" s="3"/>
       <c r="K5" s="2" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
       <c r="X5" s="2" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="Y5" s="2">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="Z5" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AA5" s="2" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="AB5" s="2" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="87" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>28</v>
@@ -1276,229 +1232,71 @@
         <v>11</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="I6" s="3">
+        <v>22.9</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="R6" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="S6" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="T6" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="I6" s="3">
-        <v>29.9</v>
-      </c>
-      <c r="J6" s="3">
-        <v>19.899999999999999</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="O6" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="R6" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="S6" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="T6" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
       <c r="W6" s="2"/>
       <c r="X6" s="2" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="Y6" s="2">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="Z6" s="2" t="s">
         <v>29</v>
       </c>
       <c r="AA6" s="2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="AB6" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="2">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="I7" s="3">
-        <v>34.99</v>
-      </c>
-      <c r="J7" s="3"/>
-      <c r="K7" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="P7" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="T7" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="U7" s="2"/>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2"/>
-      <c r="X7" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="Y7" s="2">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="AA7" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="AB7" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="2">
-        <v>11</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I8" s="3">
-        <v>22.9</v>
-      </c>
-      <c r="J8" s="3"/>
-      <c r="K8" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="O8" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="P8" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q8" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="R8" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="S8" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="Y8" s="2">
-        <v>42</v>
-      </c>
-      <c r="Z8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="AA8" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="AB8" s="2" t="s">
-        <v>146</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrige acentuacao e adiciona produto ativo Limao Siciliano
</commit_message>
<xml_diff>
--- a/data/produtos.xlsx
+++ b/data/produtos.xlsx
@@ -9,14 +9,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produtos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,11 @@
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color theme="1"/>
       <sz val="11"/>
     </font>
@@ -74,11 +79,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -92,10 +99,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 3" xfId="2"/>
+    <cellStyle name="Normal 2 2" xfId="3"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -668,7 +683,7 @@
         </is>
       </c>
       <c r="I2" s="3" t="n">
-        <v>32.9</v>
+        <v>34.9</v>
       </c>
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="2" t="inlineStr">
@@ -761,122 +776,134 @@
       </c>
     </row>
     <row r="3" ht="58" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>nao</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>vela-aromatica-lata-nude-belluno</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Velа Aromática Belluno Essenza Lata Nude</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Pureza sofisticada em design minimalista</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>vela-aromatica-belluno-limao-siciliano</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Vela Aromática Belluno Essenza Limão Siciliano</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Frescor cítrico com toque leve e elegante</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Velas aromáticas</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Floral amadeirada</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>180 g</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>40 horas</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Vela aromática premium em lata metálica nude com acabamento elegante e minimalista.</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>A vela aromática Belluno Essenza em lata metálica nude combina design sofisticado com fragrância envolvente. Seu acabamento fosco elegante cria uma presença discreta e refinada no ambiente. Ideal para momentos de relaxamento e para compor espaços com estética contemporânea e acolhedora.</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>bergamota, chá branco, lírio do vale</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>jasmim, peônia, frésia</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>âmbar, almíscar, cedro</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Acenda sobre superfície plana e deixe a cera derreter até as bordas na primeira queima.</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>Cera vegetal premium, pavio de algodão, fragrância fina</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>vela-aromatica-lata-nude-belluno.png</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="n"/>
-      <c r="V3" s="2" t="n"/>
-      <c r="W3" s="2" t="n"/>
-      <c r="X3" s="2" t="inlineStr">
-        <is>
-          <t>BEL-012</t>
-        </is>
-      </c>
-      <c r="Y3" s="2" t="n">
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Cítrica fresca</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>90g</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>16 horas</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Vela aromática artesanal de limão siciliano, com perfume cítrico, leve e luminoso para deixar o ambiente mais fresco e agradável.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>A Vela Aromática Belluno Essenza Limão Siciliano combina o frescor cítrico do limão siciliano com uma sensação limpa e delicada para o dia a dia. Produzida artesanalmente com cera vegetal e pavio de algodão, vem em recipiente de vidro com tampa de madeira, criando uma peça simples, bonita e fácil de usar na decoração. É uma boa escolha para perfumar lavabos, quartos, salas pequenas e momentos em que você quer uma casa com aroma fresco, leve e acolhedor.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>Limão siciliano, bergamota</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>Verbena, folhas verdes</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>Musk branco, toque amadeirado suave</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>Use sobre superfície plana e resistente ao calor. Na primeira queima, deixe a cera derreter até próximo das bordas para evitar túnel. Nunca deixe a vela acesa sem supervisão.</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>Cera vegetal premium, essência aromática de limão siciliano, pavio de algodão, recipiente de vidro e tampa de madeira.</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>vela-limao-siciliano-belluno-essenza-01.png</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>vela-limao-siciliano-belluno-essenza-02.png</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>vela-limao-siciliano-belluno-essenza-03.png</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>vela-limao-siciliano-belluno-essenza-04.png</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>BE-LS-90G</t>
+        </is>
+      </c>
+      <c r="Y3" s="5" t="n">
         <v>64</v>
       </c>
-      <c r="Z3" s="2" t="inlineStr">
+      <c r="Z3" s="5" t="inlineStr">
         <is>
           <t>Novo</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>Vela Aromática Belluno Essenza em Lata Nude Premium</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr">
-        <is>
-          <t>Vela aromática premium Belluno Essenza em lata metálica nude com fragrância floral sofisticada e design elegante para ambientes refinados.</t>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>Vela Aromática Limão Siciliano Belluno Essenza | Frescor Cítrico</t>
+        </is>
+      </c>
+      <c r="AB3" s="5" t="inlineStr">
+        <is>
+          <t>Vela aromática artesanal Belluno Essenza Limão Siciliano, com perfume cítrico, fresco e leve, em vidro com tampa de madeira para perfumar e decorar ambientes.</t>
         </is>
       </c>
     </row>

</xml_diff>